<commit_message>
Added patched ODEInterfaceDiffEq and patch script
so that SedTrace can be installed with Julia 1.12 until a more permament fix
becomes available
</commit_message>
<xml_diff>
--- a/test/POC1G/model_parameter_template.POC1G.xlsx
+++ b/test/POC1G/model_parameter_template.POC1G.xlsx
@@ -15,7 +15,7 @@
   <sheets>
     <sheet name="parameters" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr fullCalcOnLoad="1" calcMode="auto"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="55">
   <si>
     <t>class</t>
   </si>
@@ -584,7 +584,7 @@
       <c r="F2" t="s">
         <v>11</v>
       </c>
-      <c r="G2">
+      <c r="G2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -605,7 +605,7 @@
       <c r="F3" t="s">
         <v>14</v>
       </c>
-      <c r="G3">
+      <c r="G3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -626,7 +626,7 @@
       <c r="F4" t="s">
         <v>17</v>
       </c>
-      <c r="G4">
+      <c r="G4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -647,7 +647,7 @@
       <c r="F5" t="s">
         <v>20</v>
       </c>
-      <c r="G5">
+      <c r="G5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -668,7 +668,7 @@
       <c r="F6" t="s">
         <v>24</v>
       </c>
-      <c r="G6">
+      <c r="G6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -689,7 +689,7 @@
       <c r="F7" t="s">
         <v>27</v>
       </c>
-      <c r="G7">
+      <c r="G7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -710,7 +710,7 @@
       <c r="F8" t="s">
         <v>30</v>
       </c>
-      <c r="G8">
+      <c r="G8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -731,7 +731,7 @@
       <c r="F9" t="s">
         <v>31</v>
       </c>
-      <c r="G9">
+      <c r="G9" t="n">
         <v>1</v>
       </c>
     </row>
@@ -752,7 +752,7 @@
       <c r="F10" t="s">
         <v>35</v>
       </c>
-      <c r="G10">
+      <c r="G10" t="n">
         <v>1</v>
       </c>
     </row>
@@ -773,7 +773,7 @@
       <c r="F11" t="s">
         <v>39</v>
       </c>
-      <c r="G11">
+      <c r="G11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -794,7 +794,7 @@
       <c r="F12" t="s">
         <v>43</v>
       </c>
-      <c r="G12">
+      <c r="G12" t="n">
         <v>1</v>
       </c>
     </row>
@@ -815,7 +815,7 @@
       <c r="F13" t="s">
         <v>47</v>
       </c>
-      <c r="G13">
+      <c r="G13" t="n">
         <v>1</v>
       </c>
     </row>
@@ -836,7 +836,7 @@
       <c r="F14" t="s">
         <v>51</v>
       </c>
-      <c r="G14">
+      <c r="G14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -855,7 +855,7 @@
       <c r="F15" t="s">
         <v>54</v>
       </c>
-      <c r="G15">
+      <c r="G15" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>